<commit_message>
fix errors in data (misspelled FV classes, dʒ instead of ɟ)
</commit_message>
<xml_diff>
--- a/data/verb_paradigms.xlsx
+++ b/data/verb_paradigms.xlsx
@@ -3330,21 +3330,9 @@
       <c r="BQ18" t="inlineStr"/>
       <c r="BR18" t="inlineStr"/>
       <c r="BS18" t="inlineStr"/>
-      <c r="BT18" t="inlineStr">
-        <is>
-          <t>dʒið</t>
-        </is>
-      </c>
-      <c r="BU18" t="inlineStr">
-        <is>
-          <t>milk</t>
-        </is>
-      </c>
-      <c r="BV18" t="inlineStr">
-        <is>
-          <t>ɔi</t>
-        </is>
-      </c>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -5234,7 +5222,7 @@
       </c>
       <c r="BV29" t="inlineStr">
         <is>
-          <t>uɔ</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6236,7 @@
       </c>
       <c r="BV34" t="inlineStr">
         <is>
-          <t>oa</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -11176,21 +11164,9 @@
       <c r="BQ54" t="inlineStr"/>
       <c r="BR54" t="inlineStr"/>
       <c r="BS54" t="inlineStr"/>
-      <c r="BT54" t="inlineStr">
-        <is>
-          <t>dʒið</t>
-        </is>
-      </c>
-      <c r="BU54" t="inlineStr">
-        <is>
-          <t>milk</t>
-        </is>
-      </c>
-      <c r="BV54" t="inlineStr">
-        <is>
-          <t>ɔi</t>
-        </is>
-      </c>
+      <c r="BT54" t="inlineStr"/>
+      <c r="BU54" t="inlineStr"/>
+      <c r="BV54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -12536,7 +12512,7 @@
       </c>
       <c r="BV60" t="inlineStr">
         <is>
-          <t>oa</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19742,7 @@
       </c>
       <c r="BV89" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32199,7 @@
       </c>
       <c r="BV140" t="inlineStr">
         <is>
-          <t>uɔ</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -45045,17 +45021,17 @@
       <c r="BS224" t="inlineStr"/>
       <c r="BT224" t="inlineStr">
         <is>
-          <t>bəɽalu</t>
+          <t>biɽ</t>
         </is>
       </c>
       <c r="BU224" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>hit</t>
         </is>
       </c>
       <c r="BV224" t="inlineStr">
         <is>
-          <t>??</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -49713,7 +49689,7 @@
       </c>
       <c r="BV262" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49835,7 +49811,7 @@
       </c>
       <c r="BV263" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49969,7 +49945,7 @@
       </c>
       <c r="BV264" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50481,7 +50457,7 @@
       </c>
       <c r="BV268" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50737,7 +50713,7 @@
       </c>
       <c r="BV270" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50859,7 +50835,7 @@
       </c>
       <c r="BV271" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50975,7 +50951,7 @@
       </c>
       <c r="BV272" t="inlineStr">
         <is>
-          <t>ɔɽ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -59015,7 +58991,7 @@
       </c>
       <c r="BV330" t="inlineStr">
         <is>
-          <t>uɔ</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>

</xml_diff>